<commit_message>
swm-workbook: regenerate Minnesota Ave sample with nested-IF formulas
</commit_message>
<xml_diff>
--- a/SW_Required_Provided_DOEE_EISA438_SAMPLE_MinnesotaAve.xlsx
+++ b/SW_Required_Provided_DOEE_EISA438_SAMPLE_MinnesotaAve.xlsx
@@ -9754,11 +9754,11 @@
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4">
-        <f>IFERROR(IF(OR(E4="Enhanced",E4="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E4="Enhanced",E4="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J4" s="17">
-        <f>IFERROR(IFS(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,5),AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,5),AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K4" s="17">
@@ -9787,21 +9787,21 @@
         <v>2</v>
       </c>
       <c r="R4" s="17">
-        <f>IFERROR(IFS(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,3),AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,3),AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S4" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="T4" s="17">
-        <f>IFERROR(IFS(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,4),AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,4),AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U4" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="V4" s="4">
-        <f>IFERROR(IF(OR(E4="Enhanced",E4="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E4="Enhanced",E4="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C4,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W4" s="17">
@@ -9833,7 +9833,7 @@
         <v/>
       </c>
       <c r="AJ4" s="17">
-        <f>IFERROR(IFS(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,6),AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,6),AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D4="Permeable Pavement",E4="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D4="Permeable Pavement",E4="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D4="Bioretention",E4="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D4="Bioretention",E4="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D4="Bioretention",E4="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D4="Dry Swale",E4="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D4="Wet Swale",E4="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK4" s="17">
@@ -9883,11 +9883,11 @@
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4">
-        <f>IFERROR(IF(OR(E5="Enhanced",E5="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E5="Enhanced",E5="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J5" s="17">
-        <f>IFERROR(IFS(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,5),AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,5),AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K5" s="17">
@@ -9910,17 +9910,17 @@
       </c>
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="17">
-        <f>IFERROR(IFS(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,3),AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,3),AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S5" s="4" t="n"/>
       <c r="T5" s="17">
-        <f>IFERROR(IFS(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,4),AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,4),AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U5" s="4" t="n"/>
       <c r="V5" s="4">
-        <f>IFERROR(IF(OR(E5="Enhanced",E5="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E5="Enhanced",E5="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C5,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W5" s="17">
@@ -9952,7 +9952,7 @@
         <v/>
       </c>
       <c r="AJ5" s="17">
-        <f>IFERROR(IFS(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,6),AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,6),AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D5="Permeable Pavement",E5="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D5="Permeable Pavement",E5="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D5="Bioretention",E5="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D5="Bioretention",E5="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D5="Bioretention",E5="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D5="Dry Swale",E5="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D5="Wet Swale",E5="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK5" s="17">
@@ -10002,11 +10002,11 @@
       </c>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4">
-        <f>IFERROR(IF(OR(E6="Enhanced",E6="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E6="Enhanced",E6="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J6" s="17">
-        <f>IFERROR(IFS(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,5),AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,5),AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K6" s="17">
@@ -10029,17 +10029,17 @@
       </c>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="17">
-        <f>IFERROR(IFS(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,3),AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,3),AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S6" s="4" t="n"/>
       <c r="T6" s="17">
-        <f>IFERROR(IFS(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,4),AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,4),AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U6" s="4" t="n"/>
       <c r="V6" s="4">
-        <f>IFERROR(IF(OR(E6="Enhanced",E6="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E6="Enhanced",E6="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C6,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W6" s="17">
@@ -10071,7 +10071,7 @@
         <v/>
       </c>
       <c r="AJ6" s="17">
-        <f>IFERROR(IFS(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,6),AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,6),AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D6="Permeable Pavement",E6="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D6="Permeable Pavement",E6="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D6="Bioretention",E6="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D6="Bioretention",E6="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D6="Bioretention",E6="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D6="Dry Swale",E6="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D6="Wet Swale",E6="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK6" s="17">
@@ -10121,11 +10121,11 @@
       </c>
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4">
-        <f>IFERROR(IF(OR(E7="Enhanced",E7="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E7="Enhanced",E7="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J7" s="17">
-        <f>IFERROR(IFS(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,5),AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,5),AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K7" s="17">
@@ -10148,17 +10148,17 @@
       </c>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="17">
-        <f>IFERROR(IFS(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,3),AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,3),AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S7" s="4" t="n"/>
       <c r="T7" s="17">
-        <f>IFERROR(IFS(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,4),AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,4),AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U7" s="4" t="n"/>
       <c r="V7" s="4">
-        <f>IFERROR(IF(OR(E7="Enhanced",E7="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E7="Enhanced",E7="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C7,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W7" s="17">
@@ -10190,7 +10190,7 @@
         <v/>
       </c>
       <c r="AJ7" s="17">
-        <f>IFERROR(IFS(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,6),AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,6),AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D7="Permeable Pavement",E7="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D7="Permeable Pavement",E7="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D7="Bioretention",E7="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D7="Bioretention",E7="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D7="Bioretention",E7="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D7="Dry Swale",E7="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D7="Wet Swale",E7="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK7" s="17">
@@ -10232,11 +10232,11 @@
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4">
-        <f>IFERROR(IF(OR(E8="Enhanced",E8="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E8="Enhanced",E8="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J8" s="17">
-        <f>IFERROR(IFS(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,5),AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,5),AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K8" s="17">
@@ -10259,17 +10259,17 @@
       </c>
       <c r="Q8" s="4" t="n"/>
       <c r="R8" s="17">
-        <f>IFERROR(IFS(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,3),AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,3),AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S8" s="4" t="n"/>
       <c r="T8" s="17">
-        <f>IFERROR(IFS(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,4),AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,4),AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U8" s="4" t="n"/>
       <c r="V8" s="4">
-        <f>IFERROR(IF(OR(E8="Enhanced",E8="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E8="Enhanced",E8="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C8,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W8" s="17">
@@ -10313,7 +10313,7 @@
         <v/>
       </c>
       <c r="AJ8" s="17">
-        <f>IFERROR(IFS(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,6),AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,6),AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D8="Permeable Pavement",E8="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D8="Permeable Pavement",E8="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D8="Bioretention",E8="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D8="Bioretention",E8="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D8="Bioretention",E8="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D8="Dry Swale",E8="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D8="Wet Swale",E8="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK8" s="17">
@@ -10363,11 +10363,11 @@
       </c>
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4">
-        <f>IFERROR(IF(OR(E9="Enhanced",E9="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E9="Enhanced",E9="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J9" s="17">
-        <f>IFERROR(IFS(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,5),AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,5),AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K9" s="17">
@@ -10390,17 +10390,17 @@
       </c>
       <c r="Q9" s="4" t="n"/>
       <c r="R9" s="17">
-        <f>IFERROR(IFS(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,3),AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,3),AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S9" s="4" t="n"/>
       <c r="T9" s="17">
-        <f>IFERROR(IFS(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,4),AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,4),AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U9" s="4" t="n"/>
       <c r="V9" s="4">
-        <f>IFERROR(IF(OR(E9="Enhanced",E9="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E9="Enhanced",E9="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C9,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W9" s="17">
@@ -10432,7 +10432,7 @@
         <v/>
       </c>
       <c r="AJ9" s="17">
-        <f>IFERROR(IFS(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,6),AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,6),AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D9="Permeable Pavement",E9="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D9="Permeable Pavement",E9="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D9="Bioretention",E9="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D9="Bioretention",E9="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D9="Bioretention",E9="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D9="Dry Swale",E9="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D9="Wet Swale",E9="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK9" s="17">
@@ -10474,11 +10474,11 @@
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="4">
-        <f>IFERROR(IF(OR(E10="Enhanced",E10="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E10="Enhanced",E10="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J10" s="17">
-        <f>IFERROR(IFS(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,5),AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,5),AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K10" s="17">
@@ -10501,17 +10501,17 @@
       </c>
       <c r="Q10" s="4" t="n"/>
       <c r="R10" s="17">
-        <f>IFERROR(IFS(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,3),AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,3),AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S10" s="4" t="n"/>
       <c r="T10" s="17">
-        <f>IFERROR(IFS(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,4),AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,4),AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U10" s="4" t="n"/>
       <c r="V10" s="4">
-        <f>IFERROR(IF(OR(E10="Enhanced",E10="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E10="Enhanced",E10="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C10,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W10" s="17">
@@ -10555,7 +10555,7 @@
         <v/>
       </c>
       <c r="AJ10" s="17">
-        <f>IFERROR(IFS(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,6),AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,6),AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D10="Permeable Pavement",E10="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D10="Permeable Pavement",E10="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D10="Bioretention",E10="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D10="Bioretention",E10="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D10="Bioretention",E10="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D10="Dry Swale",E10="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D10="Wet Swale",E10="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK10" s="17">
@@ -10601,11 +10601,11 @@
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4">
-        <f>IFERROR(IF(OR(E11="Enhanced",E11="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E11="Enhanced",E11="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J11" s="17">
-        <f>IFERROR(IFS(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,5),AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,5),AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K11" s="17">
@@ -10634,21 +10634,21 @@
         <v>2</v>
       </c>
       <c r="R11" s="17">
-        <f>IFERROR(IFS(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,3),AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,3),AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S11" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="T11" s="17">
-        <f>IFERROR(IFS(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,4),AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,4),AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U11" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="V11" s="4">
-        <f>IFERROR(IF(OR(E11="Enhanced",E11="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E11="Enhanced",E11="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C11,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W11" s="17">
@@ -10680,7 +10680,7 @@
         <v/>
       </c>
       <c r="AJ11" s="17">
-        <f>IFERROR(IFS(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,6),AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,6),AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D11="Permeable Pavement",E11="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D11="Permeable Pavement",E11="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D11="Bioretention",E11="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D11="Bioretention",E11="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D11="Bioretention",E11="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D11="Dry Swale",E11="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D11="Wet Swale",E11="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK11" s="17">
@@ -10722,11 +10722,11 @@
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4">
-        <f>IFERROR(IF(OR(E12="Enhanced",E12="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E12="Enhanced",E12="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J12" s="17">
-        <f>IFERROR(IFS(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,5),AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,5),AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K12" s="17">
@@ -10749,17 +10749,17 @@
       </c>
       <c r="Q12" s="4" t="n"/>
       <c r="R12" s="17">
-        <f>IFERROR(IFS(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,3),AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,3),AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S12" s="4" t="n"/>
       <c r="T12" s="17">
-        <f>IFERROR(IFS(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,4),AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,4),AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U12" s="4" t="n"/>
       <c r="V12" s="4">
-        <f>IFERROR(IF(OR(E12="Enhanced",E12="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E12="Enhanced",E12="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C12,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W12" s="17">
@@ -10803,7 +10803,7 @@
         <v/>
       </c>
       <c r="AJ12" s="17">
-        <f>IFERROR(IFS(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,6),AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,6),AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D12="Permeable Pavement",E12="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D12="Permeable Pavement",E12="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D12="Bioretention",E12="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D12="Bioretention",E12="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D12="Bioretention",E12="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D12="Dry Swale",E12="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D12="Wet Swale",E12="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK12" s="17">
@@ -10849,11 +10849,11 @@
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4">
-        <f>IFERROR(IF(OR(E13="Enhanced",E13="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E13="Enhanced",E13="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J13" s="17">
-        <f>IFERROR(IFS(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,5),AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,5),AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K13" s="17">
@@ -10882,21 +10882,21 @@
         <v>2</v>
       </c>
       <c r="R13" s="17">
-        <f>IFERROR(IFS(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,3),AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,3),AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S13" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="T13" s="17">
-        <f>IFERROR(IFS(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,4),AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,4),AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U13" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="V13" s="4">
-        <f>IFERROR(IF(OR(E13="Enhanced",E13="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E13="Enhanced",E13="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C13,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W13" s="17">
@@ -10928,7 +10928,7 @@
         <v/>
       </c>
       <c r="AJ13" s="17">
-        <f>IFERROR(IFS(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,6),AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,6),AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D13="Permeable Pavement",E13="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D13="Permeable Pavement",E13="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D13="Bioretention",E13="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D13="Bioretention",E13="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D13="Bioretention",E13="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D13="Dry Swale",E13="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D13="Wet Swale",E13="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK13" s="17">
@@ -10970,11 +10970,11 @@
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4">
-        <f>IFERROR(IF(OR(E14="Enhanced",E14="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E14="Enhanced",E14="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J14" s="17">
-        <f>IFERROR(IFS(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,5),AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,5),AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K14" s="17">
@@ -10997,17 +10997,17 @@
       </c>
       <c r="Q14" s="4" t="n"/>
       <c r="R14" s="17">
-        <f>IFERROR(IFS(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,3),AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,3),AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S14" s="4" t="n"/>
       <c r="T14" s="17">
-        <f>IFERROR(IFS(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,4),AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,4),AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U14" s="4" t="n"/>
       <c r="V14" s="4">
-        <f>IFERROR(IF(OR(E14="Enhanced",E14="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E14="Enhanced",E14="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C14,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W14" s="17">
@@ -11051,7 +11051,7 @@
         <v/>
       </c>
       <c r="AJ14" s="17">
-        <f>IFERROR(IFS(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,6),AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,6),AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D14="Permeable Pavement",E14="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D14="Permeable Pavement",E14="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D14="Bioretention",E14="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D14="Bioretention",E14="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D14="Bioretention",E14="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D14="Dry Swale",E14="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D14="Wet Swale",E14="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK14" s="17">
@@ -11097,11 +11097,11 @@
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4">
-        <f>IFERROR(IF(OR(E15="Enhanced",E15="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E15="Enhanced",E15="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J15" s="17">
-        <f>IFERROR(IFS(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,5),AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,5),AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K15" s="17">
@@ -11130,21 +11130,21 @@
         <v>2</v>
       </c>
       <c r="R15" s="17">
-        <f>IFERROR(IFS(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,3),AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,3),AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S15" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="T15" s="17">
-        <f>IFERROR(IFS(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,4),AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,4),AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U15" s="4" t="n">
         <v>0.5</v>
       </c>
       <c r="V15" s="4">
-        <f>IFERROR(IF(OR(E15="Enhanced",E15="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E15="Enhanced",E15="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C15,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W15" s="17">
@@ -11176,7 +11176,7 @@
         <v/>
       </c>
       <c r="AJ15" s="17">
-        <f>IFERROR(IFS(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,6),AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,6),AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D15="Permeable Pavement",E15="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D15="Permeable Pavement",E15="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D15="Bioretention",E15="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D15="Bioretention",E15="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D15="Bioretention",E15="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D15="Dry Swale",E15="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D15="Wet Swale",E15="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK15" s="17">
@@ -11218,11 +11218,11 @@
       <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4">
-        <f>IFERROR(IF(OR(E16="Enhanced",E16="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E16="Enhanced",E16="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J16" s="17">
-        <f>IFERROR(IFS(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,5),AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,5),AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K16" s="17">
@@ -11245,17 +11245,17 @@
       </c>
       <c r="Q16" s="4" t="n"/>
       <c r="R16" s="17">
-        <f>IFERROR(IFS(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,3),AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,3),AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S16" s="4" t="n"/>
       <c r="T16" s="17">
-        <f>IFERROR(IFS(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,4),AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,4),AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U16" s="4" t="n"/>
       <c r="V16" s="4">
-        <f>IFERROR(IF(OR(E16="Enhanced",E16="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E16="Enhanced",E16="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C16,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W16" s="17">
@@ -11299,7 +11299,7 @@
         <v/>
       </c>
       <c r="AJ16" s="17">
-        <f>IFERROR(IFS(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,6),AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,6),AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D16="Permeable Pavement",E16="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D16="Permeable Pavement",E16="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D16="Bioretention",E16="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D16="Bioretention",E16="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D16="Bioretention",E16="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D16="Dry Swale",E16="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D16="Wet Swale",E16="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK16" s="17">
@@ -11341,11 +11341,11 @@
       <c r="G17" s="4" t="n"/>
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4">
-        <f>IFERROR(IF(OR(E17="Enhanced",E17="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E17="Enhanced",E17="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J17" s="17">
-        <f>IFERROR(IFS(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,5),AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,5),AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K17" s="17">
@@ -11368,17 +11368,17 @@
       </c>
       <c r="Q17" s="4" t="n"/>
       <c r="R17" s="17">
-        <f>IFERROR(IFS(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,3),AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,3),AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S17" s="4" t="n"/>
       <c r="T17" s="17">
-        <f>IFERROR(IFS(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,4),AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,4),AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U17" s="4" t="n"/>
       <c r="V17" s="4">
-        <f>IFERROR(IF(OR(E17="Enhanced",E17="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E17="Enhanced",E17="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C17,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W17" s="17">
@@ -11422,7 +11422,7 @@
         <v/>
       </c>
       <c r="AJ17" s="17">
-        <f>IFERROR(IFS(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,6),AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,6),AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D17="Permeable Pavement",E17="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D17="Permeable Pavement",E17="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D17="Bioretention",E17="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D17="Bioretention",E17="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D17="Bioretention",E17="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D17="Dry Swale",E17="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D17="Wet Swale",E17="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK17" s="17">
@@ -11464,11 +11464,11 @@
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4">
-        <f>IFERROR(IF(OR(E18="Enhanced",E18="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E18="Enhanced",E18="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J18" s="17">
-        <f>IFERROR(IFS(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,5),AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,5),AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K18" s="17">
@@ -11491,17 +11491,17 @@
       </c>
       <c r="Q18" s="4" t="n"/>
       <c r="R18" s="17">
-        <f>IFERROR(IFS(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,3),AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,3),AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S18" s="4" t="n"/>
       <c r="T18" s="17">
-        <f>IFERROR(IFS(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,4),AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,4),AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U18" s="4" t="n"/>
       <c r="V18" s="4">
-        <f>IFERROR(IF(OR(E18="Enhanced",E18="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E18="Enhanced",E18="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C18,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W18" s="17">
@@ -11545,7 +11545,7 @@
         <v/>
       </c>
       <c r="AJ18" s="17">
-        <f>IFERROR(IFS(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,6),AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,6),AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D18="Permeable Pavement",E18="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D18="Permeable Pavement",E18="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D18="Bioretention",E18="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D18="Bioretention",E18="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D18="Bioretention",E18="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D18="Dry Swale",E18="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D18="Wet Swale",E18="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK18" s="17">
@@ -11571,11 +11571,11 @@
       <c r="G19" s="4" t="n"/>
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4">
-        <f>IFERROR(IF(OR(E19="Enhanced",E19="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E19="Enhanced",E19="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J19" s="17">
-        <f>IFERROR(IFS(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,5),AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,5),AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K19" s="17">
@@ -11598,17 +11598,17 @@
       </c>
       <c r="Q19" s="4" t="n"/>
       <c r="R19" s="17">
-        <f>IFERROR(IFS(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,3),AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,3),AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S19" s="4" t="n"/>
       <c r="T19" s="17">
-        <f>IFERROR(IFS(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,4),AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,4),AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U19" s="4" t="n"/>
       <c r="V19" s="4">
-        <f>IFERROR(IF(OR(E19="Enhanced",E19="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E19="Enhanced",E19="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C19,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W19" s="17">
@@ -11640,7 +11640,7 @@
         <v/>
       </c>
       <c r="AJ19" s="17">
-        <f>IFERROR(IFS(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,6),AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,6),AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D19="Permeable Pavement",E19="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D19="Permeable Pavement",E19="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D19="Bioretention",E19="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D19="Bioretention",E19="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D19="Bioretention",E19="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D19="Dry Swale",E19="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D19="Wet Swale",E19="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK19" s="17">
@@ -11666,11 +11666,11 @@
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4">
-        <f>IFERROR(IF(OR(E20="Enhanced",E20="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E20="Enhanced",E20="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J20" s="17">
-        <f>IFERROR(IFS(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,5),AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,5),AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K20" s="17">
@@ -11693,17 +11693,17 @@
       </c>
       <c r="Q20" s="4" t="n"/>
       <c r="R20" s="17">
-        <f>IFERROR(IFS(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,3),AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,3),AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S20" s="4" t="n"/>
       <c r="T20" s="17">
-        <f>IFERROR(IFS(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,4),AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,4),AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U20" s="4" t="n"/>
       <c r="V20" s="4">
-        <f>IFERROR(IF(OR(E20="Enhanced",E20="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E20="Enhanced",E20="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C20,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W20" s="17">
@@ -11735,7 +11735,7 @@
         <v/>
       </c>
       <c r="AJ20" s="17">
-        <f>IFERROR(IFS(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,6),AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,6),AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D20="Permeable Pavement",E20="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D20="Permeable Pavement",E20="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D20="Bioretention",E20="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D20="Bioretention",E20="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D20="Bioretention",E20="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D20="Dry Swale",E20="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D20="Wet Swale",E20="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK20" s="17">
@@ -11761,11 +11761,11 @@
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4">
-        <f>IFERROR(IF(OR(E21="Enhanced",E21="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E21="Enhanced",E21="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J21" s="17">
-        <f>IFERROR(IFS(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,5),AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,5),AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K21" s="17">
@@ -11788,17 +11788,17 @@
       </c>
       <c r="Q21" s="4" t="n"/>
       <c r="R21" s="17">
-        <f>IFERROR(IFS(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,3),AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,3),AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S21" s="4" t="n"/>
       <c r="T21" s="17">
-        <f>IFERROR(IFS(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,4),AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,4),AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U21" s="4" t="n"/>
       <c r="V21" s="4">
-        <f>IFERROR(IF(OR(E21="Enhanced",E21="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E21="Enhanced",E21="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C21,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W21" s="17">
@@ -11830,7 +11830,7 @@
         <v/>
       </c>
       <c r="AJ21" s="17">
-        <f>IFERROR(IFS(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,6),AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,6),AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D21="Permeable Pavement",E21="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D21="Permeable Pavement",E21="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D21="Bioretention",E21="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D21="Bioretention",E21="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D21="Bioretention",E21="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D21="Dry Swale",E21="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D21="Wet Swale",E21="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK21" s="17">
@@ -11856,11 +11856,11 @@
       <c r="G22" s="4" t="n"/>
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4">
-        <f>IFERROR(IF(OR(E22="Enhanced",E22="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E22="Enhanced",E22="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J22" s="17">
-        <f>IFERROR(IFS(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,5),AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,5),AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K22" s="17">
@@ -11883,17 +11883,17 @@
       </c>
       <c r="Q22" s="4" t="n"/>
       <c r="R22" s="17">
-        <f>IFERROR(IFS(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,3),AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,3),AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S22" s="4" t="n"/>
       <c r="T22" s="17">
-        <f>IFERROR(IFS(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,4),AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,4),AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U22" s="4" t="n"/>
       <c r="V22" s="4">
-        <f>IFERROR(IF(OR(E22="Enhanced",E22="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E22="Enhanced",E22="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C22,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W22" s="17">
@@ -11925,7 +11925,7 @@
         <v/>
       </c>
       <c r="AJ22" s="17">
-        <f>IFERROR(IFS(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,6),AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,6),AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D22="Permeable Pavement",E22="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D22="Permeable Pavement",E22="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D22="Bioretention",E22="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D22="Bioretention",E22="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D22="Bioretention",E22="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D22="Dry Swale",E22="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D22="Wet Swale",E22="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK22" s="17">
@@ -11951,11 +11951,11 @@
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4">
-        <f>IFERROR(IF(OR(E23="Enhanced",E23="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E23="Enhanced",E23="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J23" s="17">
-        <f>IFERROR(IFS(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,5),AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,5),AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K23" s="17">
@@ -11978,17 +11978,17 @@
       </c>
       <c r="Q23" s="4" t="n"/>
       <c r="R23" s="17">
-        <f>IFERROR(IFS(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,3),AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,3),AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S23" s="4" t="n"/>
       <c r="T23" s="17">
-        <f>IFERROR(IFS(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,4),AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,4),AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U23" s="4" t="n"/>
       <c r="V23" s="4">
-        <f>IFERROR(IF(OR(E23="Enhanced",E23="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E23="Enhanced",E23="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C23,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W23" s="17">
@@ -12020,7 +12020,7 @@
         <v/>
       </c>
       <c r="AJ23" s="17">
-        <f>IFERROR(IFS(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,6),AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,6),AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D23="Permeable Pavement",E23="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D23="Permeable Pavement",E23="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D23="Bioretention",E23="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D23="Bioretention",E23="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D23="Bioretention",E23="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D23="Dry Swale",E23="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D23="Wet Swale",E23="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK23" s="17">
@@ -12046,11 +12046,11 @@
       <c r="G24" s="4" t="n"/>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4">
-        <f>IFERROR(IF(OR(E24="Enhanced",E24="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E24="Enhanced",E24="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J24" s="17">
-        <f>IFERROR(IFS(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,5),AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,5),AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K24" s="17">
@@ -12073,17 +12073,17 @@
       </c>
       <c r="Q24" s="4" t="n"/>
       <c r="R24" s="17">
-        <f>IFERROR(IFS(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,3),AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,3),AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S24" s="4" t="n"/>
       <c r="T24" s="17">
-        <f>IFERROR(IFS(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,4),AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,4),AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U24" s="4" t="n"/>
       <c r="V24" s="4">
-        <f>IFERROR(IF(OR(E24="Enhanced",E24="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E24="Enhanced",E24="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C24,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W24" s="17">
@@ -12115,7 +12115,7 @@
         <v/>
       </c>
       <c r="AJ24" s="17">
-        <f>IFERROR(IFS(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,6),AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,6),AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D24="Permeable Pavement",E24="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D24="Permeable Pavement",E24="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D24="Bioretention",E24="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D24="Bioretention",E24="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D24="Bioretention",E24="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D24="Dry Swale",E24="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D24="Wet Swale",E24="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK24" s="17">
@@ -12141,11 +12141,11 @@
       <c r="G25" s="4" t="n"/>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4">
-        <f>IFERROR(IF(OR(E25="Enhanced",E25="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E25="Enhanced",E25="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J25" s="17">
-        <f>IFERROR(IFS(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,5),AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,5),AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K25" s="17">
@@ -12168,17 +12168,17 @@
       </c>
       <c r="Q25" s="4" t="n"/>
       <c r="R25" s="17">
-        <f>IFERROR(IFS(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,3),AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,3),AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S25" s="4" t="n"/>
       <c r="T25" s="17">
-        <f>IFERROR(IFS(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,4),AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,4),AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U25" s="4" t="n"/>
       <c r="V25" s="4">
-        <f>IFERROR(IF(OR(E25="Enhanced",E25="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E25="Enhanced",E25="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C25,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W25" s="17">
@@ -12210,7 +12210,7 @@
         <v/>
       </c>
       <c r="AJ25" s="17">
-        <f>IFERROR(IFS(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,6),AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,6),AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D25="Permeable Pavement",E25="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D25="Permeable Pavement",E25="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D25="Bioretention",E25="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D25="Bioretention",E25="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D25="Bioretention",E25="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D25="Dry Swale",E25="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D25="Wet Swale",E25="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK25" s="17">
@@ -12236,11 +12236,11 @@
       <c r="G26" s="4" t="n"/>
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4">
-        <f>IFERROR(IF(OR(E26="Enhanced",E26="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E26="Enhanced",E26="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J26" s="17">
-        <f>IFERROR(IFS(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,5),AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,5),AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K26" s="17">
@@ -12263,17 +12263,17 @@
       </c>
       <c r="Q26" s="4" t="n"/>
       <c r="R26" s="17">
-        <f>IFERROR(IFS(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,3),AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,3),AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S26" s="4" t="n"/>
       <c r="T26" s="17">
-        <f>IFERROR(IFS(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,4),AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,4),AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U26" s="4" t="n"/>
       <c r="V26" s="4">
-        <f>IFERROR(IF(OR(E26="Enhanced",E26="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E26="Enhanced",E26="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C26,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W26" s="17">
@@ -12305,7 +12305,7 @@
         <v/>
       </c>
       <c r="AJ26" s="17">
-        <f>IFERROR(IFS(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,6),AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,6),AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D26="Permeable Pavement",E26="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D26="Permeable Pavement",E26="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D26="Bioretention",E26="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D26="Bioretention",E26="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D26="Bioretention",E26="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D26="Dry Swale",E26="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D26="Wet Swale",E26="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK26" s="17">
@@ -12331,11 +12331,11 @@
       <c r="G27" s="4" t="n"/>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4">
-        <f>IFERROR(IF(OR(E27="Enhanced",E27="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E27="Enhanced",E27="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J27" s="17">
-        <f>IFERROR(IFS(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,5),AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,5),AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K27" s="17">
@@ -12358,17 +12358,17 @@
       </c>
       <c r="Q27" s="4" t="n"/>
       <c r="R27" s="17">
-        <f>IFERROR(IFS(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,3),AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,3),AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S27" s="4" t="n"/>
       <c r="T27" s="17">
-        <f>IFERROR(IFS(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,4),AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,4),AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U27" s="4" t="n"/>
       <c r="V27" s="4">
-        <f>IFERROR(IF(OR(E27="Enhanced",E27="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E27="Enhanced",E27="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C27,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W27" s="17">
@@ -12400,7 +12400,7 @@
         <v/>
       </c>
       <c r="AJ27" s="17">
-        <f>IFERROR(IFS(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,6),AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,6),AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D27="Permeable Pavement",E27="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D27="Permeable Pavement",E27="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D27="Bioretention",E27="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D27="Bioretention",E27="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D27="Bioretention",E27="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D27="Dry Swale",E27="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D27="Wet Swale",E27="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK27" s="17">
@@ -12426,11 +12426,11 @@
       <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4">
-        <f>IFERROR(IF(OR(E28="Enhanced",E28="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E28="Enhanced",E28="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J28" s="17">
-        <f>IFERROR(IFS(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,5),AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,5),AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K28" s="17">
@@ -12453,17 +12453,17 @@
       </c>
       <c r="Q28" s="4" t="n"/>
       <c r="R28" s="17">
-        <f>IFERROR(IFS(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,3),AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,3),AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S28" s="4" t="n"/>
       <c r="T28" s="17">
-        <f>IFERROR(IFS(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,4),AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,4),AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U28" s="4" t="n"/>
       <c r="V28" s="4">
-        <f>IFERROR(IF(OR(E28="Enhanced",E28="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E28="Enhanced",E28="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C28,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W28" s="17">
@@ -12495,7 +12495,7 @@
         <v/>
       </c>
       <c r="AJ28" s="17">
-        <f>IFERROR(IFS(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,6),AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,6),AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D28="Permeable Pavement",E28="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D28="Permeable Pavement",E28="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D28="Bioretention",E28="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D28="Bioretention",E28="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D28="Bioretention",E28="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D28="Dry Swale",E28="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D28="Wet Swale",E28="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK28" s="17">
@@ -12521,11 +12521,11 @@
       <c r="G29" s="4" t="n"/>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4">
-        <f>IFERROR(IF(OR(E29="Enhanced",E29="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E29="Enhanced",E29="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J29" s="17">
-        <f>IFERROR(IFS(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,5),AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,5),AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K29" s="17">
@@ -12548,17 +12548,17 @@
       </c>
       <c r="Q29" s="4" t="n"/>
       <c r="R29" s="17">
-        <f>IFERROR(IFS(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,3),AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,3),AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S29" s="4" t="n"/>
       <c r="T29" s="17">
-        <f>IFERROR(IFS(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,4),AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,4),AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U29" s="4" t="n"/>
       <c r="V29" s="4">
-        <f>IFERROR(IF(OR(E29="Enhanced",E29="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E29="Enhanced",E29="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C29,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W29" s="17">
@@ -12590,7 +12590,7 @@
         <v/>
       </c>
       <c r="AJ29" s="17">
-        <f>IFERROR(IFS(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,6),AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,6),AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D29="Permeable Pavement",E29="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D29="Permeable Pavement",E29="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D29="Bioretention",E29="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D29="Bioretention",E29="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D29="Bioretention",E29="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D29="Dry Swale",E29="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D29="Wet Swale",E29="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK29" s="17">
@@ -12616,11 +12616,11 @@
       <c r="G30" s="4" t="n"/>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4">
-        <f>IFERROR(IF(OR(E30="Enhanced",E30="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E30="Enhanced",E30="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J30" s="17">
-        <f>IFERROR(IFS(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,5),AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,5),AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K30" s="17">
@@ -12643,17 +12643,17 @@
       </c>
       <c r="Q30" s="4" t="n"/>
       <c r="R30" s="17">
-        <f>IFERROR(IFS(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,3),AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,3),AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S30" s="4" t="n"/>
       <c r="T30" s="17">
-        <f>IFERROR(IFS(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,4),AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,4),AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U30" s="4" t="n"/>
       <c r="V30" s="4">
-        <f>IFERROR(IF(OR(E30="Enhanced",E30="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E30="Enhanced",E30="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C30,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W30" s="17">
@@ -12685,7 +12685,7 @@
         <v/>
       </c>
       <c r="AJ30" s="17">
-        <f>IFERROR(IFS(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,6),AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,6),AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D30="Permeable Pavement",E30="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D30="Permeable Pavement",E30="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D30="Bioretention",E30="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D30="Bioretention",E30="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D30="Bioretention",E30="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D30="Dry Swale",E30="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D30="Wet Swale",E30="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK30" s="17">
@@ -12711,11 +12711,11 @@
       <c r="G31" s="4" t="n"/>
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4">
-        <f>IFERROR(IF(OR(E31="Enhanced",E31="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E31="Enhanced",E31="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J31" s="17">
-        <f>IFERROR(IFS(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,5),AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,5),AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K31" s="17">
@@ -12738,17 +12738,17 @@
       </c>
       <c r="Q31" s="4" t="n"/>
       <c r="R31" s="17">
-        <f>IFERROR(IFS(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,3),AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,3),AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S31" s="4" t="n"/>
       <c r="T31" s="17">
-        <f>IFERROR(IFS(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,4),AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,4),AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U31" s="4" t="n"/>
       <c r="V31" s="4">
-        <f>IFERROR(IF(OR(E31="Enhanced",E31="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E31="Enhanced",E31="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C31,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W31" s="17">
@@ -12780,7 +12780,7 @@
         <v/>
       </c>
       <c r="AJ31" s="17">
-        <f>IFERROR(IFS(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,6),AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,6),AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D31="Permeable Pavement",E31="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D31="Permeable Pavement",E31="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D31="Bioretention",E31="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D31="Bioretention",E31="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D31="Bioretention",E31="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D31="Dry Swale",E31="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D31="Wet Swale",E31="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK31" s="17">
@@ -12806,11 +12806,11 @@
       <c r="G32" s="4" t="n"/>
       <c r="H32" s="4" t="n"/>
       <c r="I32" s="4">
-        <f>IFERROR(IF(OR(E32="Enhanced",E32="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E32="Enhanced",E32="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J32" s="17">
-        <f>IFERROR(IFS(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,5),AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,5),AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K32" s="17">
@@ -12833,17 +12833,17 @@
       </c>
       <c r="Q32" s="4" t="n"/>
       <c r="R32" s="17">
-        <f>IFERROR(IFS(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,3),AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,3),AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S32" s="4" t="n"/>
       <c r="T32" s="17">
-        <f>IFERROR(IFS(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,4),AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,4),AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U32" s="4" t="n"/>
       <c r="V32" s="4">
-        <f>IFERROR(IF(OR(E32="Enhanced",E32="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E32="Enhanced",E32="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C32,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W32" s="17">
@@ -12875,7 +12875,7 @@
         <v/>
       </c>
       <c r="AJ32" s="17">
-        <f>IFERROR(IFS(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,6),AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,6),AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D32="Permeable Pavement",E32="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D32="Permeable Pavement",E32="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D32="Bioretention",E32="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D32="Bioretention",E32="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D32="Bioretention",E32="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D32="Dry Swale",E32="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D32="Wet Swale",E32="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK32" s="17">
@@ -12901,11 +12901,11 @@
       <c r="G33" s="4" t="n"/>
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4">
-        <f>IFERROR(IF(OR(E33="Enhanced",E33="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E33="Enhanced",E33="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J33" s="17">
-        <f>IFERROR(IFS(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,5),AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,5),AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K33" s="17">
@@ -12928,17 +12928,17 @@
       </c>
       <c r="Q33" s="4" t="n"/>
       <c r="R33" s="17">
-        <f>IFERROR(IFS(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,3),AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,3),AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S33" s="4" t="n"/>
       <c r="T33" s="17">
-        <f>IFERROR(IFS(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,4),AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,4),AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U33" s="4" t="n"/>
       <c r="V33" s="4">
-        <f>IFERROR(IF(OR(E33="Enhanced",E33="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E33="Enhanced",E33="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C33,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W33" s="17">
@@ -12970,7 +12970,7 @@
         <v/>
       </c>
       <c r="AJ33" s="17">
-        <f>IFERROR(IFS(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,6),AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,6),AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D33="Permeable Pavement",E33="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D33="Permeable Pavement",E33="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D33="Bioretention",E33="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D33="Bioretention",E33="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D33="Bioretention",E33="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D33="Dry Swale",E33="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D33="Wet Swale",E33="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK33" s="17">
@@ -12996,11 +12996,11 @@
       <c r="G34" s="4" t="n"/>
       <c r="H34" s="4" t="n"/>
       <c r="I34" s="4">
-        <f>IFERROR(IF(OR(E34="Enhanced",E34="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E34="Enhanced",E34="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J34" s="17">
-        <f>IFERROR(IFS(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,5),AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,5),AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K34" s="17">
@@ -13023,17 +13023,17 @@
       </c>
       <c r="Q34" s="4" t="n"/>
       <c r="R34" s="17">
-        <f>IFERROR(IFS(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,3),AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,3),AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S34" s="4" t="n"/>
       <c r="T34" s="17">
-        <f>IFERROR(IFS(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,4),AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,4),AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U34" s="4" t="n"/>
       <c r="V34" s="4">
-        <f>IFERROR(IF(OR(E34="Enhanced",E34="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E34="Enhanced",E34="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C34,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W34" s="17">
@@ -13065,7 +13065,7 @@
         <v/>
       </c>
       <c r="AJ34" s="17">
-        <f>IFERROR(IFS(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,6),AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,6),AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D34="Permeable Pavement",E34="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D34="Permeable Pavement",E34="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D34="Bioretention",E34="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D34="Bioretention",E34="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D34="Bioretention",E34="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D34="Dry Swale",E34="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D34="Wet Swale",E34="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK34" s="17">
@@ -13091,11 +13091,11 @@
       <c r="G35" s="4" t="n"/>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4">
-        <f>IFERROR(IF(OR(E35="Enhanced",E35="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E35="Enhanced",E35="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J35" s="17">
-        <f>IFERROR(IFS(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,5),AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,5),AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K35" s="17">
@@ -13118,17 +13118,17 @@
       </c>
       <c r="Q35" s="4" t="n"/>
       <c r="R35" s="17">
-        <f>IFERROR(IFS(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,3),AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,3),AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S35" s="4" t="n"/>
       <c r="T35" s="17">
-        <f>IFERROR(IFS(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,4),AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,4),AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U35" s="4" t="n"/>
       <c r="V35" s="4">
-        <f>IFERROR(IF(OR(E35="Enhanced",E35="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E35="Enhanced",E35="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C35,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W35" s="17">
@@ -13160,7 +13160,7 @@
         <v/>
       </c>
       <c r="AJ35" s="17">
-        <f>IFERROR(IFS(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,6),AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,6),AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D35="Permeable Pavement",E35="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D35="Permeable Pavement",E35="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D35="Bioretention",E35="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D35="Bioretention",E35="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D35="Bioretention",E35="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D35="Dry Swale",E35="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D35="Wet Swale",E35="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK35" s="17">
@@ -13186,11 +13186,11 @@
       <c r="G36" s="4" t="n"/>
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4">
-        <f>IFERROR(IF(OR(E36="Enhanced",E36="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E36="Enhanced",E36="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J36" s="17">
-        <f>IFERROR(IFS(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,5),AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,5),AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K36" s="17">
@@ -13213,17 +13213,17 @@
       </c>
       <c r="Q36" s="4" t="n"/>
       <c r="R36" s="17">
-        <f>IFERROR(IFS(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,3),AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,3),AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S36" s="4" t="n"/>
       <c r="T36" s="17">
-        <f>IFERROR(IFS(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,4),AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,4),AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U36" s="4" t="n"/>
       <c r="V36" s="4">
-        <f>IFERROR(IF(OR(E36="Enhanced",E36="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E36="Enhanced",E36="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C36,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W36" s="17">
@@ -13255,7 +13255,7 @@
         <v/>
       </c>
       <c r="AJ36" s="17">
-        <f>IFERROR(IFS(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,6),AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,6),AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D36="Permeable Pavement",E36="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D36="Permeable Pavement",E36="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D36="Bioretention",E36="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D36="Bioretention",E36="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D36="Bioretention",E36="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D36="Dry Swale",E36="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D36="Wet Swale",E36="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK36" s="17">
@@ -13281,11 +13281,11 @@
       <c r="G37" s="4" t="n"/>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4">
-        <f>IFERROR(IF(OR(E37="Enhanced",E37="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E37="Enhanced",E37="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J37" s="17">
-        <f>IFERROR(IFS(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,5),AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,5),AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K37" s="17">
@@ -13308,17 +13308,17 @@
       </c>
       <c r="Q37" s="4" t="n"/>
       <c r="R37" s="17">
-        <f>IFERROR(IFS(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,3),AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,3),AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S37" s="4" t="n"/>
       <c r="T37" s="17">
-        <f>IFERROR(IFS(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,4),AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,4),AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U37" s="4" t="n"/>
       <c r="V37" s="4">
-        <f>IFERROR(IF(OR(E37="Enhanced",E37="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E37="Enhanced",E37="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C37,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W37" s="17">
@@ -13350,7 +13350,7 @@
         <v/>
       </c>
       <c r="AJ37" s="17">
-        <f>IFERROR(IFS(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,6),AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,6),AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D37="Permeable Pavement",E37="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D37="Permeable Pavement",E37="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D37="Bioretention",E37="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D37="Bioretention",E37="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D37="Bioretention",E37="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D37="Dry Swale",E37="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D37="Wet Swale",E37="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK37" s="17">
@@ -13376,11 +13376,11 @@
       <c r="G38" s="4" t="n"/>
       <c r="H38" s="4" t="n"/>
       <c r="I38" s="4">
-        <f>IFERROR(IF(OR(E38="Enhanced",E38="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E38="Enhanced",E38="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J38" s="17">
-        <f>IFERROR(IFS(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,5),AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,5),AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K38" s="17">
@@ -13403,17 +13403,17 @@
       </c>
       <c r="Q38" s="4" t="n"/>
       <c r="R38" s="17">
-        <f>IFERROR(IFS(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,3),AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,3),AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S38" s="4" t="n"/>
       <c r="T38" s="17">
-        <f>IFERROR(IFS(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,4),AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,4),AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U38" s="4" t="n"/>
       <c r="V38" s="4">
-        <f>IFERROR(IF(OR(E38="Enhanced",E38="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E38="Enhanced",E38="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C38,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W38" s="17">
@@ -13445,7 +13445,7 @@
         <v/>
       </c>
       <c r="AJ38" s="17">
-        <f>IFERROR(IFS(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,6),AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,6),AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D38="Permeable Pavement",E38="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D38="Permeable Pavement",E38="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D38="Bioretention",E38="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D38="Bioretention",E38="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D38="Bioretention",E38="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D38="Dry Swale",E38="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D38="Wet Swale",E38="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK38" s="17">
@@ -13471,11 +13471,11 @@
       <c r="G39" s="4" t="n"/>
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4">
-        <f>IFERROR(IF(OR(E39="Enhanced",E39="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E39="Enhanced",E39="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J39" s="17">
-        <f>IFERROR(IFS(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,5),AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,5),AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K39" s="17">
@@ -13498,17 +13498,17 @@
       </c>
       <c r="Q39" s="4" t="n"/>
       <c r="R39" s="17">
-        <f>IFERROR(IFS(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,3),AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,3),AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S39" s="4" t="n"/>
       <c r="T39" s="17">
-        <f>IFERROR(IFS(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,4),AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,4),AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U39" s="4" t="n"/>
       <c r="V39" s="4">
-        <f>IFERROR(IF(OR(E39="Enhanced",E39="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E39="Enhanced",E39="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C39,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W39" s="17">
@@ -13540,7 +13540,7 @@
         <v/>
       </c>
       <c r="AJ39" s="17">
-        <f>IFERROR(IFS(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,6),AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,6),AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D39="Permeable Pavement",E39="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D39="Permeable Pavement",E39="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D39="Bioretention",E39="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D39="Bioretention",E39="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D39="Bioretention",E39="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D39="Dry Swale",E39="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D39="Wet Swale",E39="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK39" s="17">
@@ -13566,11 +13566,11 @@
       <c r="G40" s="4" t="n"/>
       <c r="H40" s="4" t="n"/>
       <c r="I40" s="4">
-        <f>IFERROR(IF(OR(E40="Enhanced",E40="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E40="Enhanced",E40="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J40" s="17">
-        <f>IFERROR(IFS(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,5),AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,5),AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K40" s="17">
@@ -13593,17 +13593,17 @@
       </c>
       <c r="Q40" s="4" t="n"/>
       <c r="R40" s="17">
-        <f>IFERROR(IFS(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,3),AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,3),AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S40" s="4" t="n"/>
       <c r="T40" s="17">
-        <f>IFERROR(IFS(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,4),AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,4),AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U40" s="4" t="n"/>
       <c r="V40" s="4">
-        <f>IFERROR(IF(OR(E40="Enhanced",E40="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E40="Enhanced",E40="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C40,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W40" s="17">
@@ -13635,7 +13635,7 @@
         <v/>
       </c>
       <c r="AJ40" s="17">
-        <f>IFERROR(IFS(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,6),AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,6),AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D40="Permeable Pavement",E40="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D40="Permeable Pavement",E40="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D40="Bioretention",E40="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D40="Bioretention",E40="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D40="Bioretention",E40="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D40="Dry Swale",E40="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D40="Wet Swale",E40="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK40" s="17">
@@ -13661,11 +13661,11 @@
       <c r="G41" s="4" t="n"/>
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4">
-        <f>IFERROR(IF(OR(E41="Enhanced",E41="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E41="Enhanced",E41="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J41" s="17">
-        <f>IFERROR(IFS(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,5),AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,5),AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K41" s="17">
@@ -13688,17 +13688,17 @@
       </c>
       <c r="Q41" s="4" t="n"/>
       <c r="R41" s="17">
-        <f>IFERROR(IFS(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,3),AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,3),AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S41" s="4" t="n"/>
       <c r="T41" s="17">
-        <f>IFERROR(IFS(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,4),AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,4),AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U41" s="4" t="n"/>
       <c r="V41" s="4">
-        <f>IFERROR(IF(OR(E41="Enhanced",E41="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E41="Enhanced",E41="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C41,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W41" s="17">
@@ -13730,7 +13730,7 @@
         <v/>
       </c>
       <c r="AJ41" s="17">
-        <f>IFERROR(IFS(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,6),AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,6),AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D41="Permeable Pavement",E41="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D41="Permeable Pavement",E41="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D41="Bioretention",E41="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D41="Bioretention",E41="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D41="Bioretention",E41="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D41="Dry Swale",E41="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D41="Wet Swale",E41="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK41" s="17">
@@ -13756,11 +13756,11 @@
       <c r="G42" s="4" t="n"/>
       <c r="H42" s="4" t="n"/>
       <c r="I42" s="4">
-        <f>IFERROR(IF(OR(E42="Enhanced",E42="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E42="Enhanced",E42="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J42" s="17">
-        <f>IFERROR(IFS(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,5),AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,5),AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K42" s="17">
@@ -13783,17 +13783,17 @@
       </c>
       <c r="Q42" s="4" t="n"/>
       <c r="R42" s="17">
-        <f>IFERROR(IFS(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,3),AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,3),AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S42" s="4" t="n"/>
       <c r="T42" s="17">
-        <f>IFERROR(IFS(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,4),AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,4),AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U42" s="4" t="n"/>
       <c r="V42" s="4">
-        <f>IFERROR(IF(OR(E42="Enhanced",E42="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E42="Enhanced",E42="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C42,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W42" s="17">
@@ -13825,7 +13825,7 @@
         <v/>
       </c>
       <c r="AJ42" s="17">
-        <f>IFERROR(IFS(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,6),AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,6),AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D42="Permeable Pavement",E42="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D42="Permeable Pavement",E42="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D42="Bioretention",E42="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D42="Bioretention",E42="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D42="Bioretention",E42="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D42="Dry Swale",E42="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D42="Wet Swale",E42="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK42" s="17">
@@ -13851,11 +13851,11 @@
       <c r="G43" s="4" t="n"/>
       <c r="H43" s="4" t="n"/>
       <c r="I43" s="4">
-        <f>IFERROR(IF(OR(E43="Enhanced",E43="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E43="Enhanced",E43="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J43" s="17">
-        <f>IFERROR(IFS(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,5),AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,5),AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K43" s="17">
@@ -13878,17 +13878,17 @@
       </c>
       <c r="Q43" s="4" t="n"/>
       <c r="R43" s="17">
-        <f>IFERROR(IFS(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,3),AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,3),AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S43" s="4" t="n"/>
       <c r="T43" s="17">
-        <f>IFERROR(IFS(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,4),AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,4),AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U43" s="4" t="n"/>
       <c r="V43" s="4">
-        <f>IFERROR(IF(OR(E43="Enhanced",E43="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E43="Enhanced",E43="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C43,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W43" s="17">
@@ -13920,7 +13920,7 @@
         <v/>
       </c>
       <c r="AJ43" s="17">
-        <f>IFERROR(IFS(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,6),AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,6),AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D43="Permeable Pavement",E43="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D43="Permeable Pavement",E43="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D43="Bioretention",E43="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D43="Bioretention",E43="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D43="Bioretention",E43="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D43="Dry Swale",E43="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D43="Wet Swale",E43="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK43" s="17">
@@ -13946,11 +13946,11 @@
       <c r="G44" s="4" t="n"/>
       <c r="H44" s="4" t="n"/>
       <c r="I44" s="4">
-        <f>IFERROR(IF(OR(E44="Enhanced",E44="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E44="Enhanced",E44="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J44" s="17">
-        <f>IFERROR(IFS(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,5),AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,5),AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K44" s="17">
@@ -13973,17 +13973,17 @@
       </c>
       <c r="Q44" s="4" t="n"/>
       <c r="R44" s="17">
-        <f>IFERROR(IFS(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,3),AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,3),AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S44" s="4" t="n"/>
       <c r="T44" s="17">
-        <f>IFERROR(IFS(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,4),AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,4),AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U44" s="4" t="n"/>
       <c r="V44" s="4">
-        <f>IFERROR(IF(OR(E44="Enhanced",E44="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E44="Enhanced",E44="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C44,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W44" s="17">
@@ -14015,7 +14015,7 @@
         <v/>
       </c>
       <c r="AJ44" s="17">
-        <f>IFERROR(IFS(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,6),AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,6),AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D44="Permeable Pavement",E44="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D44="Permeable Pavement",E44="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D44="Bioretention",E44="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D44="Bioretention",E44="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D44="Bioretention",E44="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D44="Dry Swale",E44="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D44="Wet Swale",E44="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK44" s="17">
@@ -14041,11 +14041,11 @@
       <c r="G45" s="4" t="n"/>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4">
-        <f>IFERROR(IF(OR(E45="Enhanced",E45="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E45="Enhanced",E45="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J45" s="17">
-        <f>IFERROR(IFS(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,5),AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,5),AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K45" s="17">
@@ -14068,17 +14068,17 @@
       </c>
       <c r="Q45" s="4" t="n"/>
       <c r="R45" s="17">
-        <f>IFERROR(IFS(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,3),AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,3),AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S45" s="4" t="n"/>
       <c r="T45" s="17">
-        <f>IFERROR(IFS(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,4),AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,4),AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U45" s="4" t="n"/>
       <c r="V45" s="4">
-        <f>IFERROR(IF(OR(E45="Enhanced",E45="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E45="Enhanced",E45="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C45,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W45" s="17">
@@ -14110,7 +14110,7 @@
         <v/>
       </c>
       <c r="AJ45" s="17">
-        <f>IFERROR(IFS(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,6),AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,6),AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D45="Permeable Pavement",E45="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D45="Permeable Pavement",E45="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D45="Bioretention",E45="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D45="Bioretention",E45="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D45="Bioretention",E45="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D45="Dry Swale",E45="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D45="Wet Swale",E45="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK45" s="17">
@@ -14136,11 +14136,11 @@
       <c r="G46" s="4" t="n"/>
       <c r="H46" s="4" t="n"/>
       <c r="I46" s="4">
-        <f>IFERROR(IF(OR(E46="Enhanced",E46="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E46="Enhanced",E46="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J46" s="17">
-        <f>IFERROR(IFS(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,5),AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,5),AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K46" s="17">
@@ -14163,17 +14163,17 @@
       </c>
       <c r="Q46" s="4" t="n"/>
       <c r="R46" s="17">
-        <f>IFERROR(IFS(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,3),AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,3),AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S46" s="4" t="n"/>
       <c r="T46" s="17">
-        <f>IFERROR(IFS(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,4),AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,4),AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U46" s="4" t="n"/>
       <c r="V46" s="4">
-        <f>IFERROR(IF(OR(E46="Enhanced",E46="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E46="Enhanced",E46="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C46,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W46" s="17">
@@ -14205,7 +14205,7 @@
         <v/>
       </c>
       <c r="AJ46" s="17">
-        <f>IFERROR(IFS(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,6),AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,6),AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D46="Permeable Pavement",E46="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D46="Permeable Pavement",E46="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D46="Bioretention",E46="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D46="Bioretention",E46="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D46="Bioretention",E46="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D46="Dry Swale",E46="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D46="Wet Swale",E46="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK46" s="17">
@@ -14231,11 +14231,11 @@
       <c r="G47" s="4" t="n"/>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4">
-        <f>IFERROR(IF(OR(E47="Enhanced",E47="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E47="Enhanced",E47="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J47" s="17">
-        <f>IFERROR(IFS(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,5),AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,5),AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K47" s="17">
@@ -14258,17 +14258,17 @@
       </c>
       <c r="Q47" s="4" t="n"/>
       <c r="R47" s="17">
-        <f>IFERROR(IFS(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,3),AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,3),AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S47" s="4" t="n"/>
       <c r="T47" s="17">
-        <f>IFERROR(IFS(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,4),AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,4),AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U47" s="4" t="n"/>
       <c r="V47" s="4">
-        <f>IFERROR(IF(OR(E47="Enhanced",E47="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E47="Enhanced",E47="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C47,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W47" s="17">
@@ -14300,7 +14300,7 @@
         <v/>
       </c>
       <c r="AJ47" s="17">
-        <f>IFERROR(IFS(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,6),AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,6),AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D47="Permeable Pavement",E47="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D47="Permeable Pavement",E47="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D47="Bioretention",E47="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D47="Bioretention",E47="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D47="Bioretention",E47="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D47="Dry Swale",E47="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D47="Wet Swale",E47="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK47" s="17">
@@ -14326,11 +14326,11 @@
       <c r="G48" s="4" t="n"/>
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4">
-        <f>IFERROR(IF(OR(E48="Enhanced",E48="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E48="Enhanced",E48="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J48" s="17">
-        <f>IFERROR(IFS(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,5),AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,5),AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K48" s="17">
@@ -14353,17 +14353,17 @@
       </c>
       <c r="Q48" s="4" t="n"/>
       <c r="R48" s="17">
-        <f>IFERROR(IFS(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,3),AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,3),AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S48" s="4" t="n"/>
       <c r="T48" s="17">
-        <f>IFERROR(IFS(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,4),AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,4),AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U48" s="4" t="n"/>
       <c r="V48" s="4">
-        <f>IFERROR(IF(OR(E48="Enhanced",E48="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E48="Enhanced",E48="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C48,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W48" s="17">
@@ -14395,7 +14395,7 @@
         <v/>
       </c>
       <c r="AJ48" s="17">
-        <f>IFERROR(IFS(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,6),AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,6),AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D48="Permeable Pavement",E48="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D48="Permeable Pavement",E48="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D48="Bioretention",E48="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D48="Bioretention",E48="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D48="Bioretention",E48="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D48="Dry Swale",E48="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D48="Wet Swale",E48="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK48" s="17">
@@ -14421,11 +14421,11 @@
       <c r="G49" s="4" t="n"/>
       <c r="H49" s="4" t="n"/>
       <c r="I49" s="4">
-        <f>IFERROR(IF(OR(E49="Enhanced",E49="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E49="Enhanced",E49="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J49" s="17">
-        <f>IFERROR(IFS(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,5),AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,5),AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K49" s="17">
@@ -14448,17 +14448,17 @@
       </c>
       <c r="Q49" s="4" t="n"/>
       <c r="R49" s="17">
-        <f>IFERROR(IFS(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,3),AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,3),AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S49" s="4" t="n"/>
       <c r="T49" s="17">
-        <f>IFERROR(IFS(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,4),AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,4),AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U49" s="4" t="n"/>
       <c r="V49" s="4">
-        <f>IFERROR(IF(OR(E49="Enhanced",E49="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E49="Enhanced",E49="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C49,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W49" s="17">
@@ -14490,7 +14490,7 @@
         <v/>
       </c>
       <c r="AJ49" s="17">
-        <f>IFERROR(IFS(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,6),AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,6),AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D49="Permeable Pavement",E49="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D49="Permeable Pavement",E49="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D49="Bioretention",E49="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D49="Bioretention",E49="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D49="Bioretention",E49="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D49="Dry Swale",E49="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D49="Wet Swale",E49="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK49" s="17">
@@ -14516,11 +14516,11 @@
       <c r="G50" s="4" t="n"/>
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4">
-        <f>IFERROR(IF(OR(E50="Enhanced",E50="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E50="Enhanced",E50="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J50" s="17">
-        <f>IFERROR(IFS(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,5),AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,5),AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K50" s="17">
@@ -14543,17 +14543,17 @@
       </c>
       <c r="Q50" s="4" t="n"/>
       <c r="R50" s="17">
-        <f>IFERROR(IFS(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,3),AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,3),AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S50" s="4" t="n"/>
       <c r="T50" s="17">
-        <f>IFERROR(IFS(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,4),AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,4),AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U50" s="4" t="n"/>
       <c r="V50" s="4">
-        <f>IFERROR(IF(OR(E50="Enhanced",E50="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E50="Enhanced",E50="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C50,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W50" s="17">
@@ -14585,7 +14585,7 @@
         <v/>
       </c>
       <c r="AJ50" s="17">
-        <f>IFERROR(IFS(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,6),AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,6),AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D50="Permeable Pavement",E50="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D50="Permeable Pavement",E50="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D50="Bioretention",E50="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D50="Bioretention",E50="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D50="Bioretention",E50="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D50="Dry Swale",E50="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D50="Wet Swale",E50="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK50" s="17">
@@ -14611,11 +14611,11 @@
       <c r="G51" s="4" t="n"/>
       <c r="H51" s="4" t="n"/>
       <c r="I51" s="4">
-        <f>IFERROR(IF(OR(E51="Enhanced",E51="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E51="Enhanced",E51="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J51" s="17">
-        <f>IFERROR(IFS(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,5),AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,5),AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K51" s="17">
@@ -14638,17 +14638,17 @@
       </c>
       <c r="Q51" s="4" t="n"/>
       <c r="R51" s="17">
-        <f>IFERROR(IFS(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,3),AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,3),AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S51" s="4" t="n"/>
       <c r="T51" s="17">
-        <f>IFERROR(IFS(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,4),AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,4),AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U51" s="4" t="n"/>
       <c r="V51" s="4">
-        <f>IFERROR(IF(OR(E51="Enhanced",E51="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E51="Enhanced",E51="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C51,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W51" s="17">
@@ -14680,7 +14680,7 @@
         <v/>
       </c>
       <c r="AJ51" s="17">
-        <f>IFERROR(IFS(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,6),AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,6),AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D51="Permeable Pavement",E51="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D51="Permeable Pavement",E51="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D51="Bioretention",E51="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D51="Bioretention",E51="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D51="Bioretention",E51="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D51="Dry Swale",E51="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D51="Wet Swale",E51="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK51" s="17">
@@ -14706,11 +14706,11 @@
       <c r="G52" s="4" t="n"/>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4">
-        <f>IFERROR(IF(OR(E52="Enhanced",E52="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E52="Enhanced",E52="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J52" s="17">
-        <f>IFERROR(IFS(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,5),AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,5),AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K52" s="17">
@@ -14733,17 +14733,17 @@
       </c>
       <c r="Q52" s="4" t="n"/>
       <c r="R52" s="17">
-        <f>IFERROR(IFS(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,3),AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,3),AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S52" s="4" t="n"/>
       <c r="T52" s="17">
-        <f>IFERROR(IFS(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,4),AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,4),AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U52" s="4" t="n"/>
       <c r="V52" s="4">
-        <f>IFERROR(IF(OR(E52="Enhanced",E52="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E52="Enhanced",E52="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C52,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W52" s="17">
@@ -14775,7 +14775,7 @@
         <v/>
       </c>
       <c r="AJ52" s="17">
-        <f>IFERROR(IFS(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,6),AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,6),AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D52="Permeable Pavement",E52="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D52="Permeable Pavement",E52="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D52="Bioretention",E52="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D52="Bioretention",E52="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D52="Bioretention",E52="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D52="Dry Swale",E52="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D52="Wet Swale",E52="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK52" s="17">
@@ -14801,11 +14801,11 @@
       <c r="G53" s="4" t="n"/>
       <c r="H53" s="4" t="n"/>
       <c r="I53" s="4">
-        <f>IFERROR(IF(OR(E53="Enhanced",E53="Underdrained Enhanced"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E53="Enhanced",E53="Underdrained Enhanced"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="J53" s="17">
-        <f>IFERROR(IFS(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,5),AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,5),AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,5),AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,5),AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,5),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,5),IF(AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,5),IF(AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,5),IF(AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,5),IF(AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,5),IF(AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,5),IF(AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,5),""))))))),"")</f>
         <v/>
       </c>
       <c r="K53" s="17">
@@ -14828,17 +14828,17 @@
       </c>
       <c r="Q53" s="4" t="n"/>
       <c r="R53" s="17">
-        <f>IFERROR(IFS(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,3),AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,3),AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,3),AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,3),AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,3),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,3),IF(AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,3),IF(AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,3),IF(AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,3),IF(AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,3),IF(AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,3),IF(AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,3),""))))))),"")</f>
         <v/>
       </c>
       <c r="S53" s="4" t="n"/>
       <c r="T53" s="17">
-        <f>IFERROR(IFS(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,4),AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,4),AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,4),AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,4),AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,4),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,4),IF(AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,4),IF(AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,4),IF(AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,4),IF(AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,4),IF(AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,4),IF(AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,4),""))))))),"")</f>
         <v/>
       </c>
       <c r="U53" s="4" t="n"/>
       <c r="V53" s="4">
-        <f>IFERROR(IF(OR(E53="Enhanced",E53="Enhanced w/ Underdrain"),VLOOKUP(IFS(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),PARAMS_Ksat,2,FALSE),0),0)</f>
+        <f>IFERROR(IF(OR(E53="Enhanced",E53="Enhanced w/ Underdrain"),VLOOKUP(IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('CDA'!$E$4:$E$53,'CDA'!$A$4:$A$53,C53,'CDA'!$D$4:$D$53,"A")&gt;0,"A","")))),PARAMS_Ksat,2,FALSE),0),0)</f>
         <v/>
       </c>
       <c r="W53" s="17">
@@ -14870,7 +14870,7 @@
         <v/>
       </c>
       <c r="AJ53" s="17">
-        <f>IFERROR(IFS(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,6),AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,6),AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,6),AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,6),AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,6),TRUE,""),"")</f>
+        <f>IFERROR(IF(AND(D53="Permeable Pavement",E53="Enhanced"),INDEX(PARAMS_BMP,1,6),IF(AND(D53="Permeable Pavement",E53="Underdrained Enhanced"),INDEX(PARAMS_BMP,2,6),IF(AND(D53="Bioretention",E53="Standard"),INDEX(PARAMS_BMP,3,6),IF(AND(D53="Bioretention",E53="Enhanced"),INDEX(PARAMS_BMP,4,6),IF(AND(D53="Bioretention",E53="Enhanced w/ Underdrain"),INDEX(PARAMS_BMP,5,6),IF(AND(D53="Dry Swale",E53="—"),INDEX(PARAMS_BMP,6,6),IF(AND(D53="Wet Swale",E53="—"),INDEX(PARAMS_BMP,7,6),""))))))),"")</f>
         <v/>
       </c>
       <c r="AK53" s="17">
@@ -16098,7 +16098,7 @@
         <v/>
       </c>
       <c r="L12" s="17">
-        <f>IF(A12="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A12="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A12,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M12" s="4" t="inlineStr">
@@ -16112,7 +16112,7 @@
         </is>
       </c>
       <c r="O12" s="17">
-        <f>IF(A12="","",IFS(L12="A",2.5,L12="B",0.3,L12="C",0.1,L12="D",0.05,TRUE,""))</f>
+        <f>IF(A12="","",IF(L12="A",2.5,IF(L12="B",0.3,IF(L12="C",0.1,IF(L12="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P12" s="27" t="inlineStr">
@@ -16255,7 +16255,7 @@
         <v/>
       </c>
       <c r="L13" s="17">
-        <f>IF(A13="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A13="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A13,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M13" s="4" t="inlineStr">
@@ -16269,7 +16269,7 @@
         </is>
       </c>
       <c r="O13" s="17">
-        <f>IF(A13="","",IFS(L13="A",2.5,L13="B",0.3,L13="C",0.1,L13="D",0.05,TRUE,""))</f>
+        <f>IF(A13="","",IF(L13="A",2.5,IF(L13="B",0.3,IF(L13="C",0.1,IF(L13="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P13" s="27" t="inlineStr">
@@ -16412,7 +16412,7 @@
         <v/>
       </c>
       <c r="L14" s="17">
-        <f>IF(A14="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A14="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A14,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M14" s="4" t="inlineStr">
@@ -16426,7 +16426,7 @@
         </is>
       </c>
       <c r="O14" s="17">
-        <f>IF(A14="","",IFS(L14="A",2.5,L14="B",0.3,L14="C",0.1,L14="D",0.05,TRUE,""))</f>
+        <f>IF(A14="","",IF(L14="A",2.5,IF(L14="B",0.3,IF(L14="C",0.1,IF(L14="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P14" s="27" t="inlineStr">
@@ -16569,7 +16569,7 @@
         <v/>
       </c>
       <c r="L15" s="17">
-        <f>IF(A15="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A15="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A15,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M15" s="4" t="inlineStr">
@@ -16583,7 +16583,7 @@
         </is>
       </c>
       <c r="O15" s="17">
-        <f>IF(A15="","",IFS(L15="A",2.5,L15="B",0.3,L15="C",0.1,L15="D",0.05,TRUE,""))</f>
+        <f>IF(A15="","",IF(L15="A",2.5,IF(L15="B",0.3,IF(L15="C",0.1,IF(L15="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P15" s="27" t="inlineStr">
@@ -16726,7 +16726,7 @@
         <v/>
       </c>
       <c r="L16" s="17">
-        <f>IF(A16="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A16="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A16,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -16740,7 +16740,7 @@
         </is>
       </c>
       <c r="O16" s="17">
-        <f>IF(A16="","",IFS(L16="A",2.5,L16="B",0.3,L16="C",0.1,L16="D",0.05,TRUE,""))</f>
+        <f>IF(A16="","",IF(L16="A",2.5,IF(L16="B",0.3,IF(L16="C",0.1,IF(L16="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P16" s="27" t="inlineStr">
@@ -16883,7 +16883,7 @@
         <v/>
       </c>
       <c r="L17" s="17">
-        <f>IF(A17="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A17="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A17,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -16897,7 +16897,7 @@
         </is>
       </c>
       <c r="O17" s="17">
-        <f>IF(A17="","",IFS(L17="A",2.5,L17="B",0.3,L17="C",0.1,L17="D",0.05,TRUE,""))</f>
+        <f>IF(A17="","",IF(L17="A",2.5,IF(L17="B",0.3,IF(L17="C",0.1,IF(L17="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P17" s="27" t="inlineStr">
@@ -17040,7 +17040,7 @@
         <v/>
       </c>
       <c r="L18" s="17">
-        <f>IF(A18="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A18="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A18,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M18" s="4" t="inlineStr">
@@ -17054,7 +17054,7 @@
         </is>
       </c>
       <c r="O18" s="17">
-        <f>IF(A18="","",IFS(L18="A",2.5,L18="B",0.3,L18="C",0.1,L18="D",0.05,TRUE,""))</f>
+        <f>IF(A18="","",IF(L18="A",2.5,IF(L18="B",0.3,IF(L18="C",0.1,IF(L18="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P18" s="27" t="inlineStr">
@@ -17197,7 +17197,7 @@
         <v/>
       </c>
       <c r="L19" s="17">
-        <f>IF(A19="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A19="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A19,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M19" s="4" t="inlineStr">
@@ -17211,7 +17211,7 @@
         </is>
       </c>
       <c r="O19" s="17">
-        <f>IF(A19="","",IFS(L19="A",2.5,L19="B",0.3,L19="C",0.1,L19="D",0.05,TRUE,""))</f>
+        <f>IF(A19="","",IF(L19="A",2.5,IF(L19="B",0.3,IF(L19="C",0.1,IF(L19="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P19" s="27" t="inlineStr">
@@ -17354,7 +17354,7 @@
         <v/>
       </c>
       <c r="L20" s="17">
-        <f>IF(A20="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A20="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A20,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M20" s="4" t="inlineStr">
@@ -17368,7 +17368,7 @@
         </is>
       </c>
       <c r="O20" s="17">
-        <f>IF(A20="","",IFS(L20="A",2.5,L20="B",0.3,L20="C",0.1,L20="D",0.05,TRUE,""))</f>
+        <f>IF(A20="","",IF(L20="A",2.5,IF(L20="B",0.3,IF(L20="C",0.1,IF(L20="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P20" s="27" t="inlineStr">
@@ -17511,7 +17511,7 @@
         <v/>
       </c>
       <c r="L21" s="17">
-        <f>IF(A21="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A21="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A21,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M21" s="4" t="inlineStr">
@@ -17525,7 +17525,7 @@
         </is>
       </c>
       <c r="O21" s="17">
-        <f>IF(A21="","",IFS(L21="A",2.5,L21="B",0.3,L21="C",0.1,L21="D",0.05,TRUE,""))</f>
+        <f>IF(A21="","",IF(L21="A",2.5,IF(L21="B",0.3,IF(L21="C",0.1,IF(L21="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P21" s="27" t="inlineStr">
@@ -17668,13 +17668,13 @@
         <v/>
       </c>
       <c r="L22" s="17">
-        <f>IF(A22="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A22="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A22,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M22" s="4" t="n"/>
       <c r="N22" s="4" t="n"/>
       <c r="O22" s="17">
-        <f>IF(A22="","",IFS(L22="A",2.5,L22="B",0.3,L22="C",0.1,L22="D",0.05,TRUE,""))</f>
+        <f>IF(A22="","",IF(L22="A",2.5,IF(L22="B",0.3,IF(L22="C",0.1,IF(L22="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P22" s="27" t="n"/>
@@ -17813,13 +17813,13 @@
         <v/>
       </c>
       <c r="L23" s="17">
-        <f>IF(A23="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A23="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A23,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M23" s="4" t="n"/>
       <c r="N23" s="4" t="n"/>
       <c r="O23" s="17">
-        <f>IF(A23="","",IFS(L23="A",2.5,L23="B",0.3,L23="C",0.1,L23="D",0.05,TRUE,""))</f>
+        <f>IF(A23="","",IF(L23="A",2.5,IF(L23="B",0.3,IF(L23="C",0.1,IF(L23="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P23" s="27" t="n"/>
@@ -17958,13 +17958,13 @@
         <v/>
       </c>
       <c r="L24" s="17">
-        <f>IF(A24="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A24="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A24,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M24" s="4" t="n"/>
       <c r="N24" s="4" t="n"/>
       <c r="O24" s="17">
-        <f>IF(A24="","",IFS(L24="A",2.5,L24="B",0.3,L24="C",0.1,L24="D",0.05,TRUE,""))</f>
+        <f>IF(A24="","",IF(L24="A",2.5,IF(L24="B",0.3,IF(L24="C",0.1,IF(L24="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P24" s="27" t="n"/>
@@ -18103,13 +18103,13 @@
         <v/>
       </c>
       <c r="L25" s="17">
-        <f>IF(A25="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A25="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A25,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M25" s="4" t="n"/>
       <c r="N25" s="4" t="n"/>
       <c r="O25" s="17">
-        <f>IF(A25="","",IFS(L25="A",2.5,L25="B",0.3,L25="C",0.1,L25="D",0.05,TRUE,""))</f>
+        <f>IF(A25="","",IF(L25="A",2.5,IF(L25="B",0.3,IF(L25="C",0.1,IF(L25="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P25" s="27" t="n"/>
@@ -18248,13 +18248,13 @@
         <v/>
       </c>
       <c r="L26" s="17">
-        <f>IF(A26="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A26="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A26,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M26" s="4" t="n"/>
       <c r="N26" s="4" t="n"/>
       <c r="O26" s="17">
-        <f>IF(A26="","",IFS(L26="A",2.5,L26="B",0.3,L26="C",0.1,L26="D",0.05,TRUE,""))</f>
+        <f>IF(A26="","",IF(L26="A",2.5,IF(L26="B",0.3,IF(L26="C",0.1,IF(L26="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P26" s="27" t="n"/>
@@ -18393,13 +18393,13 @@
         <v/>
       </c>
       <c r="L27" s="17">
-        <f>IF(A27="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A27="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A27,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M27" s="4" t="n"/>
       <c r="N27" s="4" t="n"/>
       <c r="O27" s="17">
-        <f>IF(A27="","",IFS(L27="A",2.5,L27="B",0.3,L27="C",0.1,L27="D",0.05,TRUE,""))</f>
+        <f>IF(A27="","",IF(L27="A",2.5,IF(L27="B",0.3,IF(L27="C",0.1,IF(L27="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P27" s="27" t="n"/>
@@ -18538,13 +18538,13 @@
         <v/>
       </c>
       <c r="L28" s="17">
-        <f>IF(A28="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A28="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A28,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M28" s="4" t="n"/>
       <c r="N28" s="4" t="n"/>
       <c r="O28" s="17">
-        <f>IF(A28="","",IFS(L28="A",2.5,L28="B",0.3,L28="C",0.1,L28="D",0.05,TRUE,""))</f>
+        <f>IF(A28="","",IF(L28="A",2.5,IF(L28="B",0.3,IF(L28="C",0.1,IF(L28="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P28" s="27" t="n"/>
@@ -18683,13 +18683,13 @@
         <v/>
       </c>
       <c r="L29" s="17">
-        <f>IF(A29="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A29="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A29,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M29" s="4" t="n"/>
       <c r="N29" s="4" t="n"/>
       <c r="O29" s="17">
-        <f>IF(A29="","",IFS(L29="A",2.5,L29="B",0.3,L29="C",0.1,L29="D",0.05,TRUE,""))</f>
+        <f>IF(A29="","",IF(L29="A",2.5,IF(L29="B",0.3,IF(L29="C",0.1,IF(L29="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P29" s="27" t="n"/>
@@ -18828,13 +18828,13 @@
         <v/>
       </c>
       <c r="L30" s="17">
-        <f>IF(A30="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A30="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A30,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M30" s="4" t="n"/>
       <c r="N30" s="4" t="n"/>
       <c r="O30" s="17">
-        <f>IF(A30="","",IFS(L30="A",2.5,L30="B",0.3,L30="C",0.1,L30="D",0.05,TRUE,""))</f>
+        <f>IF(A30="","",IF(L30="A",2.5,IF(L30="B",0.3,IF(L30="C",0.1,IF(L30="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P30" s="27" t="n"/>
@@ -18973,13 +18973,13 @@
         <v/>
       </c>
       <c r="L31" s="17">
-        <f>IF(A31="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A31="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A31,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M31" s="4" t="n"/>
       <c r="N31" s="4" t="n"/>
       <c r="O31" s="17">
-        <f>IF(A31="","",IFS(L31="A",2.5,L31="B",0.3,L31="C",0.1,L31="D",0.05,TRUE,""))</f>
+        <f>IF(A31="","",IF(L31="A",2.5,IF(L31="B",0.3,IF(L31="C",0.1,IF(L31="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P31" s="27" t="n"/>
@@ -19118,13 +19118,13 @@
         <v/>
       </c>
       <c r="L32" s="17">
-        <f>IF(A32="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A32="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A32,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M32" s="4" t="n"/>
       <c r="N32" s="4" t="n"/>
       <c r="O32" s="17">
-        <f>IF(A32="","",IFS(L32="A",2.5,L32="B",0.3,L32="C",0.1,L32="D",0.05,TRUE,""))</f>
+        <f>IF(A32="","",IF(L32="A",2.5,IF(L32="B",0.3,IF(L32="C",0.1,IF(L32="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P32" s="27" t="n"/>
@@ -19263,13 +19263,13 @@
         <v/>
       </c>
       <c r="L33" s="17">
-        <f>IF(A33="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A33="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A33,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M33" s="4" t="n"/>
       <c r="N33" s="4" t="n"/>
       <c r="O33" s="17">
-        <f>IF(A33="","",IFS(L33="A",2.5,L33="B",0.3,L33="C",0.1,L33="D",0.05,TRUE,""))</f>
+        <f>IF(A33="","",IF(L33="A",2.5,IF(L33="B",0.3,IF(L33="C",0.1,IF(L33="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P33" s="27" t="n"/>
@@ -19408,13 +19408,13 @@
         <v/>
       </c>
       <c r="L34" s="17">
-        <f>IF(A34="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A34="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A34,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M34" s="4" t="n"/>
       <c r="N34" s="4" t="n"/>
       <c r="O34" s="17">
-        <f>IF(A34="","",IFS(L34="A",2.5,L34="B",0.3,L34="C",0.1,L34="D",0.05,TRUE,""))</f>
+        <f>IF(A34="","",IF(L34="A",2.5,IF(L34="B",0.3,IF(L34="C",0.1,IF(L34="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P34" s="27" t="n"/>
@@ -19553,13 +19553,13 @@
         <v/>
       </c>
       <c r="L35" s="17">
-        <f>IF(A35="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A35="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A35,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M35" s="4" t="n"/>
       <c r="N35" s="4" t="n"/>
       <c r="O35" s="17">
-        <f>IF(A35="","",IFS(L35="A",2.5,L35="B",0.3,L35="C",0.1,L35="D",0.05,TRUE,""))</f>
+        <f>IF(A35="","",IF(L35="A",2.5,IF(L35="B",0.3,IF(L35="C",0.1,IF(L35="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P35" s="27" t="n"/>
@@ -19698,13 +19698,13 @@
         <v/>
       </c>
       <c r="L36" s="17">
-        <f>IF(A36="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A36="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A36,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M36" s="4" t="n"/>
       <c r="N36" s="4" t="n"/>
       <c r="O36" s="17">
-        <f>IF(A36="","",IFS(L36="A",2.5,L36="B",0.3,L36="C",0.1,L36="D",0.05,TRUE,""))</f>
+        <f>IF(A36="","",IF(L36="A",2.5,IF(L36="B",0.3,IF(L36="C",0.1,IF(L36="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P36" s="27" t="n"/>
@@ -19843,13 +19843,13 @@
         <v/>
       </c>
       <c r="L37" s="17">
-        <f>IF(A37="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A37="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A37,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M37" s="4" t="n"/>
       <c r="N37" s="4" t="n"/>
       <c r="O37" s="17">
-        <f>IF(A37="","",IFS(L37="A",2.5,L37="B",0.3,L37="C",0.1,L37="D",0.05,TRUE,""))</f>
+        <f>IF(A37="","",IF(L37="A",2.5,IF(L37="B",0.3,IF(L37="C",0.1,IF(L37="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P37" s="27" t="n"/>
@@ -19988,13 +19988,13 @@
         <v/>
       </c>
       <c r="L38" s="17">
-        <f>IF(A38="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A38="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A38,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M38" s="4" t="n"/>
       <c r="N38" s="4" t="n"/>
       <c r="O38" s="17">
-        <f>IF(A38="","",IFS(L38="A",2.5,L38="B",0.3,L38="C",0.1,L38="D",0.05,TRUE,""))</f>
+        <f>IF(A38="","",IF(L38="A",2.5,IF(L38="B",0.3,IF(L38="C",0.1,IF(L38="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P38" s="27" t="n"/>
@@ -20133,13 +20133,13 @@
         <v/>
       </c>
       <c r="L39" s="17">
-        <f>IF(A39="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A39="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A39,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M39" s="4" t="n"/>
       <c r="N39" s="4" t="n"/>
       <c r="O39" s="17">
-        <f>IF(A39="","",IFS(L39="A",2.5,L39="B",0.3,L39="C",0.1,L39="D",0.05,TRUE,""))</f>
+        <f>IF(A39="","",IF(L39="A",2.5,IF(L39="B",0.3,IF(L39="C",0.1,IF(L39="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P39" s="27" t="n"/>
@@ -20278,13 +20278,13 @@
         <v/>
       </c>
       <c r="L40" s="17">
-        <f>IF(A40="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A40="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A40,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M40" s="4" t="n"/>
       <c r="N40" s="4" t="n"/>
       <c r="O40" s="17">
-        <f>IF(A40="","",IFS(L40="A",2.5,L40="B",0.3,L40="C",0.1,L40="D",0.05,TRUE,""))</f>
+        <f>IF(A40="","",IF(L40="A",2.5,IF(L40="B",0.3,IF(L40="C",0.1,IF(L40="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P40" s="27" t="n"/>
@@ -20423,13 +20423,13 @@
         <v/>
       </c>
       <c r="L41" s="17">
-        <f>IF(A41="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A41="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A41,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M41" s="4" t="n"/>
       <c r="N41" s="4" t="n"/>
       <c r="O41" s="17">
-        <f>IF(A41="","",IFS(L41="A",2.5,L41="B",0.3,L41="C",0.1,L41="D",0.05,TRUE,""))</f>
+        <f>IF(A41="","",IF(L41="A",2.5,IF(L41="B",0.3,IF(L41="C",0.1,IF(L41="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P41" s="27" t="n"/>
@@ -20568,13 +20568,13 @@
         <v/>
       </c>
       <c r="L42" s="17">
-        <f>IF(A42="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A42="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A42,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M42" s="4" t="n"/>
       <c r="N42" s="4" t="n"/>
       <c r="O42" s="17">
-        <f>IF(A42="","",IFS(L42="A",2.5,L42="B",0.3,L42="C",0.1,L42="D",0.05,TRUE,""))</f>
+        <f>IF(A42="","",IF(L42="A",2.5,IF(L42="B",0.3,IF(L42="C",0.1,IF(L42="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P42" s="27" t="n"/>
@@ -20713,13 +20713,13 @@
         <v/>
       </c>
       <c r="L43" s="17">
-        <f>IF(A43="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A43="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A43,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M43" s="4" t="n"/>
       <c r="N43" s="4" t="n"/>
       <c r="O43" s="17">
-        <f>IF(A43="","",IFS(L43="A",2.5,L43="B",0.3,L43="C",0.1,L43="D",0.05,TRUE,""))</f>
+        <f>IF(A43="","",IF(L43="A",2.5,IF(L43="B",0.3,IF(L43="C",0.1,IF(L43="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P43" s="27" t="n"/>
@@ -20858,13 +20858,13 @@
         <v/>
       </c>
       <c r="L44" s="17">
-        <f>IF(A44="","",IFERROR(IFS(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"D")&gt;0,"D",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"C")&gt;0,"C",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"B")&gt;0,"B",SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"A")&gt;0,"A",TRUE,""),""))</f>
+        <f>IF(A44="","",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"D")&gt;0,"D",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"C")&gt;0,"C",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"B")&gt;0,"B",IF(SUMIFS('SDA'!$G$4:$G$53,'SDA'!$A$4:$A$53,A44,'SDA'!$D$4:$D$53,"A")&gt;0,"A","")))))</f>
         <v/>
       </c>
       <c r="M44" s="4" t="n"/>
       <c r="N44" s="4" t="n"/>
       <c r="O44" s="17">
-        <f>IF(A44="","",IFS(L44="A",2.5,L44="B",0.3,L44="C",0.1,L44="D",0.05,TRUE,""))</f>
+        <f>IF(A44="","",IF(L44="A",2.5,IF(L44="B",0.3,IF(L44="C",0.1,IF(L44="D",0.05,"")))))</f>
         <v/>
       </c>
       <c r="P44" s="27" t="n"/>

</xml_diff>